<commit_message>
Added stagger map outputs with HST comparison. Also added Rayleigh-Kuo Criterion for Barotropic Instability.
</commit_message>
<xml_diff>
--- a/windfield_datarecords.xlsx
+++ b/windfield_datarecords.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahyder/Desktop/windfieldproject/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93A601CB-EFC0-1C4B-B8E4-55C9F9FE6986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{776C8916-52FB-5348-B930-070341BADDFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14780" yWindow="4860" windowWidth="34560" windowHeight="19880" activeTab="1" xr2:uid="{42A9C88B-2997-EB4C-AFF6-033636F0CE16}"/>
+    <workbookView xWindow="0" yWindow="880" windowWidth="34560" windowHeight="19880" activeTab="1" xr2:uid="{42A9C88B-2997-EB4C-AFF6-033636F0CE16}"/>
   </bookViews>
   <sheets>
     <sheet name="5µ" sheetId="1" r:id="rId1"/>
@@ -8472,6 +8472,9 @@
       <c r="B108" s="1" t="s">
         <v>1302</v>
       </c>
+      <c r="C108" s="18" t="s">
+        <v>714</v>
+      </c>
       <c r="D108" s="17">
         <v>5</v>
       </c>
@@ -8491,9 +8494,6 @@
       </c>
       <c r="B109" t="s">
         <v>1287</v>
-      </c>
-      <c r="C109" s="18" t="s">
-        <v>714</v>
       </c>
       <c r="D109" s="17">
         <v>5</v>

</xml_diff>